<commit_message>
Retire the old-format sign-off sets of BRD-02, BRD-03, BRD-06 and BRD-11: the FRS in BDOI's format and its review workbooks are the only documents
The four set folders are removed from the drops (38 files). brand.py maps the retired BRDs to their BDOI-format pack (BDOI_FRS_SETS, RETIRED_SETS, refuse_retired); the sign-off, test plan, guide deck, UX deck and configuration input builders refuse these BRDs without --force; check_pack refuses a retired folder that reappears or a missing BDOI-format FRS; the drop indexes and the Drop 0 closure summary point to the BDOI-format pack. Closure set v2.1 rebuilt (new seed tables listed as records, employees, legacy accounts and payees claimed, CCM and MFT parameter wording); BRD-04 and BRD-05 test plans rebuilt with the BRD-02 test cases and traceability workbook as their reference.
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Drop-1_Transactional/BRD-04_Collections/04_BIBS_TestPlan_BRD-04_Collections_v2.1.xlsx
+++ b/docs/deliverables/out/Drop-1_Transactional/BRD-04_Collections/04_BIBS_TestPlan_BRD-04_Collections_v2.1.xlsx
@@ -34037,9 +34037,9 @@
       <c r="L275" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-CL-009: "Invoice &lt;invoice no&gt; is paid directly to the insurer / cancelled and has no premium to collect" (CLX_INVOICE_NOT_COLLECTIBLE)
-MSG-CL-010: "Invoice &lt;invoice no&gt; is not in the ledger" (CLX_INVOICE_UNKNOWN)
-MSG-CL-011: "&lt;editing by&gt; is editing &lt;invoice no&gt;" (CLX_ITEM_LOCKED)</t>
+MSG-CL-010: "Invoice &lt;invoice no&gt; is paid directly to the insurer / cancelled and has no premium to collect" (CLX_INVOICE_NOT_COLLECTIBLE)
+MSG-CL-011: "Invoice &lt;invoice no&gt; is not in the ledger" (CLX_INVOICE_UNKNOWN)
+MSG-CL-012: "&lt;editing by&gt; is editing &lt;invoice no&gt;" (CLX_ITEM_LOCKED)</t>
         </is>
       </c>
       <c r="M275" s="12" t="inlineStr">
@@ -34114,22 +34114,22 @@
       <c r="L276" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-CL-012: "A certificate tag needs the certificate number"
-MSG-CL-013: "Check pick-up"
-MSG-CL-014: "Choose a disposition"
-MSG-CL-015: "The pick-up date cannot be in the past"
-MSG-CL-016: "You are not allowed to update several accounts at once" (CLX_BULK_NOT_ALLOWED)
-MSG-CL-017: "The tagging category is A, B or C" (CLX_CATEGORY)
-MSG-CL-018: "Choose the 2307 path: certificate received or paid in cash" (CLX_CWT_PATH)
-MSG-CL-019: "'&lt;v&gt;' is not a date (yyyy-mm-dd)" (CLX_DISPOSITION_DETAIL)
-MSG-CL-020: "'&lt;v&gt;' is not an amount" (CLX_DISPOSITION_DETAIL)
-MSG-CL-021: "Give &lt;what&gt;" (CLX_DISPOSITION_DETAIL)
-MSG-CL-022: "This disposition is reserved to other roles" (CLX_DISPOSITION_NOT_ALLOWED)
-MSG-CL-023: "An effort cannot be in the future" (CLX_EFFORT_FUTURE)
-MSG-CL-024: "&lt;invoice no&gt; is &lt;status&gt;" (CLX_ITEM_CLOSED)
-MSG-CL-025: "&lt;invoice no&gt; belongs to another company" (CLX_ITEM_OTHER_COMPANY)
-MSG-CL-026: "Select at least one account" (CLX_NO_ACCOUNT)
-MSG-CL-027: "Select at most 500 accounts at once" (CLX_TOO_MANY_ACCOUNTS)</t>
+MSG-CL-013: "A certificate tag needs the certificate number"
+MSG-CL-014: "Check pick-up"
+MSG-CL-015: "Choose a disposition"
+MSG-CL-016: "The pick-up date cannot be in the past"
+MSG-CL-017: "You are not allowed to update several accounts at once" (CLX_BULK_NOT_ALLOWED)
+MSG-CL-018: "The tagging category is A, B or C" (CLX_CATEGORY)
+MSG-CL-019: "Choose the 2307 path: certificate received or paid in cash" (CLX_CWT_PATH)
+MSG-CL-020: "'&lt;v&gt;' is not a date (yyyy-mm-dd)" (CLX_DISPOSITION_DETAIL)
+MSG-CL-021: "'&lt;v&gt;' is not an amount" (CLX_DISPOSITION_DETAIL)
+MSG-CL-022: "Give &lt;what&gt;" (CLX_DISPOSITION_DETAIL)
+MSG-CL-023: "This disposition is reserved to other roles" (CLX_DISPOSITION_NOT_ALLOWED)
+MSG-CL-024: "An effort cannot be in the future" (CLX_EFFORT_FUTURE)
+MSG-CL-025: "&lt;invoice no&gt; is &lt;status&gt;" (CLX_ITEM_CLOSED)
+MSG-CL-026: "&lt;invoice no&gt; belongs to another company" (CLX_ITEM_OTHER_COMPANY)
+MSG-CL-027: "Select at least one account" (CLX_NO_ACCOUNT)
+MSG-CL-028: "Select at most 500 accounts at once" (CLX_TOO_MANY_ACCOUNTS)</t>
         </is>
       </c>
       <c r="M276" s="12" t="inlineStr">
@@ -34204,15 +34204,15 @@
       <c r="L277" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-CL-037: "Plan &lt;plan no&gt; has no billing cycle &lt;seq&gt;" (CLX_CYCLE_UNKNOWN)
-MSG-CL-038: "Billing frequency &lt;code&gt; has no cycle length defined" (CLX_FREQUENCY_UNSUPPORTED)
-MSG-CL-039: "A plan needs at least one installment" (CLX_PLAN_EMPTY)
-MSG-CL-040: "Enter at least one installment" (CLX_PLAN_EMPTY)
-MSG-CL-041: "Installment amounts must be positive and due dates increasing" (CLX_PLAN_ENTRY_INVALID)
-MSG-CL-042: "Plan &lt;plan no&gt; already schedules this account; cancel it first" (CLX_PLAN_EXISTS)
-MSG-CL-043: "Invoice &lt;invoice no&gt; has no outstanding premium to schedule" (CLX_PLAN_NOTHING_DUE)
-MSG-CL-044: "Plan &lt;plan no&gt; is &lt;status&gt; and cannot be cancelled" (CLX_PLAN_NOT_ACTIVE)
-MSG-CL-045: "Account &lt;arn&gt; has no booked policy year" (CLX_PLAN_NOT_BOOKED)</t>
+MSG-CL-038: "Plan &lt;plan no&gt; has no billing cycle &lt;seq&gt;" (CLX_CYCLE_UNKNOWN)
+MSG-CL-039: "Billing frequency &lt;code&gt; has no cycle length defined" (CLX_FREQUENCY_UNSUPPORTED)
+MSG-CL-040: "A plan needs at least one installment" (CLX_PLAN_EMPTY)
+MSG-CL-041: "Enter at least one installment" (CLX_PLAN_EMPTY)
+MSG-CL-042: "Installment amounts must be positive and due dates increasing" (CLX_PLAN_ENTRY_INVALID)
+MSG-CL-043: "Plan &lt;plan no&gt; already schedules this account; cancel it first" (CLX_PLAN_EXISTS)
+MSG-CL-044: "Invoice &lt;invoice no&gt; has no outstanding premium to schedule" (CLX_PLAN_NOTHING_DUE)
+MSG-CL-045: "Plan &lt;plan no&gt; is &lt;status&gt; and cannot be cancelled" (CLX_PLAN_NOT_ACTIVE)
+MSG-CL-046: "Account &lt;arn&gt; has no booked policy year" (CLX_PLAN_NOT_BOOKED)</t>
         </is>
       </c>
       <c r="M277" s="12" t="inlineStr">
@@ -34287,12 +34287,12 @@
       <c r="L278" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-CL-050: "The promised amount must be positive" (CLX_PROMISE_AMOUNT)
-MSG-CL-051: "The promise of &lt;invoice no&gt; is already &lt;status&gt;" (CLX_PROMISE_CLOSED)
-MSG-CL-052: "Enter the promised date; the day of the promise cannot be in the future" (CLX_PROMISE_DATES)
-MSG-CL-053: "The promised date cannot be before the day of the promise" (CLX_PROMISE_DATES)
-MSG-CL-054: "The installment does not bill invoice &lt;invoice no&gt;" (CLX_PROMISE_INSTALLMENT)
-MSG-CL-055: "Invoice &lt;invoice no&gt; has nothing to collect" (CLX_PROMISE_NOTHING_DUE)</t>
+MSG-CL-051: "The promised amount must be positive" (CLX_PROMISE_AMOUNT)
+MSG-CL-052: "The promise of &lt;invoice no&gt; is already &lt;status&gt;" (CLX_PROMISE_CLOSED)
+MSG-CL-053: "Enter the promised date; the day of the promise cannot be in the future" (CLX_PROMISE_DATES)
+MSG-CL-054: "The promised date cannot be before the day of the promise" (CLX_PROMISE_DATES)
+MSG-CL-055: "The installment does not bill invoice &lt;invoice no&gt;" (CLX_PROMISE_INSTALLMENT)
+MSG-CL-056: "Invoice &lt;invoice no&gt; has nothing to collect" (CLX_PROMISE_NOTHING_DUE)</t>
         </is>
       </c>
       <c r="M278" s="12" t="inlineStr">
@@ -34355,7 +34355,7 @@
       <c r="L279" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-CL-056: "Enter the &lt;label&gt;"</t>
+MSG-CL-057: "Enter the &lt;label&gt;"</t>
         </is>
       </c>
       <c r="M279" s="12" t="inlineStr">
@@ -34430,9 +34430,9 @@
       <c r="L280" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-CL-059: "Plan &lt;plan no&gt; is cancelled" (CLX_PLAN_NOT_ACTIVE)
-MSG-CL-060: "Cycle &lt;cycle seq&gt; of &lt;plan no&gt; is billed by &lt;soa no&gt;" (CLX_SOA_EXISTS)
-MSG-CL-061: "The period ends before it starts" (CLX_SOA_PERIOD)</t>
+MSG-CL-060: "Plan &lt;plan no&gt; is cancelled" (CLX_PLAN_NOT_ACTIVE)
+MSG-CL-061: "Cycle &lt;cycle seq&gt; of &lt;plan no&gt; is billed by &lt;soa no&gt;" (CLX_SOA_EXISTS)
+MSG-CL-062: "The period ends before it starts" (CLX_SOA_PERIOD)</t>
         </is>
       </c>
       <c r="M280" s="12" t="inlineStr">
@@ -34507,8 +34507,8 @@
       <c r="L281" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-CL-062: "Statement &lt;soa no&gt; is cancelled" (CLX_SOA_CANCELLED)
-MSG-CL-063: "Enter at least one recipient" (CLX_SOA_RECIPIENT)</t>
+MSG-CL-063: "Statement &lt;soa no&gt; is cancelled" (CLX_SOA_CANCELLED)
+MSG-CL-064: "Enter at least one recipient" (CLX_SOA_RECIPIENT)</t>
         </is>
       </c>
       <c r="M281" s="12" t="inlineStr">
@@ -34583,10 +34583,10 @@
       <c r="L282" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-CL-065: "'&lt;action&gt;' is not an escalation action" (CLX_ESCALATION_ACTION)
-MSG-CL-066: "&lt;username&gt; does not handle escalations" (CLX_ESCALATION_TARGET)
-MSG-CL-067: "Choose the level, and the user for a designated authority" (CLX_ESCALATION_TARGET)
-MSG-CL-068: "Describe how the escalation was resolved" (CLX_RESOLUTION_REQUIRED)</t>
+MSG-CL-066: "'&lt;action&gt;' is not an escalation action" (CLX_ESCALATION_ACTION)
+MSG-CL-067: "&lt;username&gt; does not handle escalations" (CLX_ESCALATION_TARGET)
+MSG-CL-068: "Choose the level, and the user for a designated authority" (CLX_ESCALATION_TARGET)
+MSG-CL-069: "Describe how the escalation was resolved" (CLX_RESOLUTION_REQUIRED)</t>
         </is>
       </c>
       <c r="M282" s="12" t="inlineStr">
@@ -34661,12 +34661,12 @@
       <c r="L283" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-CL-071: "The amount range ends below its start" (CLX_RULE_AMOUNTS)
-MSG-CL-072: "Enter the company and the rule code" (CLX_RULE_CODE)
-MSG-CL-073: "The rule cannot end before it becomes effective" (CLX_RULE_DATES)
-MSG-CL-074: "The threshold and the SLA hours must be positive" (CLX_RULE_INVALID)
-MSG-CL-075: "Name the user who receives the escalations of this rule" (CLX_RULE_TARGET)
-MSG-CL-076: "Escalation rule already exists: &lt;key&gt;" (DUPLICATE)</t>
+MSG-CL-072: "The amount range ends below its start" (CLX_RULE_AMOUNTS)
+MSG-CL-073: "Enter the company and the rule code" (CLX_RULE_CODE)
+MSG-CL-074: "The rule cannot end before it becomes effective" (CLX_RULE_DATES)
+MSG-CL-075: "The threshold and the SLA hours must be positive" (CLX_RULE_INVALID)
+MSG-CL-076: "Name the user who receives the escalations of this rule" (CLX_RULE_TARGET)
+MSG-CL-077: "Escalation rule already exists: &lt;key&gt;" (DUPLICATE)</t>
         </is>
       </c>
       <c r="M283" s="12" t="inlineStr">
@@ -34741,10 +34741,10 @@
       <c r="L284" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-CL-078: "Invoice number &lt;clean&gt; does not have the expected format (&lt;invoice pattern&gt;)" (CLX_INVOICE_FORMAT)
-MSG-CL-079: "Enter the invoice number to apply the payment to" (CLX_INVOICE_REQUIRED)
-MSG-CL-080: "Invoice &lt;clean&gt; is not in the invoice ledger" (CLX_INVOICE_UNKNOWN)
-MSG-CL-081: "&lt;unapplied ref&gt; has no unapplied balance left" (CLX_UNAPPLIED_NO_BALANCE)</t>
+MSG-CL-079: "Invoice number &lt;clean&gt; does not have the expected format (&lt;invoice pattern&gt;)" (CLX_INVOICE_FORMAT)
+MSG-CL-080: "Enter the invoice number to apply the payment to" (CLX_INVOICE_REQUIRED)
+MSG-CL-081: "Invoice &lt;clean&gt; is not in the invoice ledger" (CLX_INVOICE_UNKNOWN)
+MSG-CL-082: "&lt;unapplied ref&gt; has no unapplied balance left" (CLX_UNAPPLIED_NO_BALANCE)</t>
         </is>
       </c>
       <c r="M284" s="12" t="inlineStr">
@@ -34819,13 +34819,13 @@
       <c r="L285" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-CL-090: "&lt;handler&gt; is not an active collection handler" (CLX_HANDLER_NOT_ELIGIBLE)
-MSG-CL-091: "No account matches the selection" (CLX_REASSIGN_EMPTY)
-MSG-CL-092: "A temporary reassignment needs an end date after today" (CLX_REASSIGN_END_DATE)
-MSG-CL-093: "Choose a permanent or a temporary reassignment" (CLX_REASSIGN_KIND)
-MSG-CL-094: "Give the reason of the reassignment" (CLX_REASSIGN_REASON)
-MSG-CL-095: "Give the rule a name" (CLX_RULE_NAME)
-MSG-CL-096: "A range must start before it ends" (CLX_RULE_RANGE)</t>
+MSG-CL-091: "&lt;handler&gt; is not an active collection handler" (CLX_HANDLER_NOT_ELIGIBLE)
+MSG-CL-092: "No account matches the selection" (CLX_REASSIGN_EMPTY)
+MSG-CL-093: "A temporary reassignment needs an end date after today" (CLX_REASSIGN_END_DATE)
+MSG-CL-094: "Choose a permanent or a temporary reassignment" (CLX_REASSIGN_KIND)
+MSG-CL-095: "Give the reason of the reassignment" (CLX_REASSIGN_REASON)
+MSG-CL-096: "Give the rule a name" (CLX_RULE_NAME)
+MSG-CL-097: "A range must start before it ends" (CLX_RULE_RANGE)</t>
         </is>
       </c>
       <c r="M285" s="12" t="inlineStr">
@@ -34900,14 +34900,14 @@
       <c r="L286" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-CL-098: "The aging basis is BOOKING or INCEPTION" (CLX_AGING_BASIS)
-MSG-CL-099: "Aging bracket '&lt;text&gt;' ends before it starts" (CLX_AGING_BRACKETS_INVALID)
-MSG-CL-100: "Aging bracket '&lt;text&gt;' is not from-to or from+" (CLX_AGING_BRACKETS_INVALID)
-MSG-CL-101: "Aging brackets must be in ascending order: &lt;raw&gt;" (CLX_AGING_BRACKETS_INVALID)
-MSG-CL-102: "&lt;attribute&gt; is not an attribute of &lt;type code&gt;" (CLX_LOV_ATTRIBUTE_UNKNOWN)
-MSG-CL-103: "'&lt;value&gt;' is not a valid &lt;attribute&gt;" (CLX_LOV_ATTRIBUTE_VALUE)
-MSG-CL-104: "&lt;code&gt; is not a value of &lt;type code&gt;" (CLX_LOV_VALUE_UNKNOWN)
-MSG-CL-105: "&lt;key&gt; is not a Collections parameter" (CLX_PARAMETER_NOT_COLLECTIONS)</t>
+MSG-CL-099: "The aging basis is BOOKING or INCEPTION" (CLX_AGING_BASIS)
+MSG-CL-100: "Aging bracket '&lt;text&gt;' ends before it starts" (CLX_AGING_BRACKETS_INVALID)
+MSG-CL-101: "Aging bracket '&lt;text&gt;' is not from-to or from+" (CLX_AGING_BRACKETS_INVALID)
+MSG-CL-102: "Aging brackets must be in ascending order: &lt;raw&gt;" (CLX_AGING_BRACKETS_INVALID)
+MSG-CL-103: "&lt;attribute&gt; is not an attribute of &lt;type code&gt;" (CLX_LOV_ATTRIBUTE_UNKNOWN)
+MSG-CL-104: "'&lt;value&gt;' is not a valid &lt;attribute&gt;" (CLX_LOV_ATTRIBUTE_VALUE)
+MSG-CL-105: "&lt;code&gt; is not a value of &lt;type code&gt;" (CLX_LOV_VALUE_UNKNOWN)
+MSG-CL-106: "&lt;key&gt; is not a Collections parameter" (CLX_PARAMETER_NOT_COLLECTIONS)</t>
         </is>
       </c>
       <c r="M286" s="12" t="inlineStr">
@@ -34970,29 +34970,29 @@
       <c r="L287" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-CL-106: "Choose the billing frequency"
-MSG-CL-107: "Choose the disposition"
-MSG-CL-108: "Choose the escalation reason"
-MSG-CL-109: "Enter a positive amount, or leave it empty for the whole outstanding"
-MSG-CL-110: "Enter a positive threshold"
-MSG-CL-111: "Enter an amount above zero and at most &lt;balance&gt;"
-MSG-CL-112: "Enter at least one invoice number"
-MSG-CL-113: "Enter between 1 and 120 installments"
-MSG-CL-114: "Enter between 1 and 720 hours"
-MSG-CL-115: "Enter both dates"
-MSG-CL-116: "Enter the account reference number"
-MSG-CL-117: "Enter the first day"
-MSG-CL-118: "Enter the first due date"
-MSG-CL-119: "Enter the invoice number"
-MSG-CL-120: "Enter the invoice number to apply the payment to"
-MSG-CL-121: "Enter the promised payment date"
-MSG-CL-122: "Enter the rule code"
-MSG-CL-123: "Enter the rule name"
-MSG-CL-124: "Name the user who receives the escalations"
-MSG-CL-125: "The day of the promise cannot be in the future"
-MSG-CL-126: "The invoice number does not have the expected format"
-MSG-CL-127: "The promised date cannot be before the day of the promise"
-MSG-CL-128: "The rule cannot end before it starts"</t>
+MSG-CL-107: "Choose the billing frequency"
+MSG-CL-108: "Choose the disposition"
+MSG-CL-109: "Choose the escalation reason"
+MSG-CL-110: "Enter a positive amount, or leave it empty for the whole outstanding"
+MSG-CL-111: "Enter a positive threshold"
+MSG-CL-112: "Enter an amount above zero and at most &lt;balance&gt;"
+MSG-CL-113: "Enter at least one invoice number"
+MSG-CL-114: "Enter between 1 and 120 installments"
+MSG-CL-115: "Enter between 1 and 720 hours"
+MSG-CL-116: "Enter both dates"
+MSG-CL-117: "Enter the account reference number"
+MSG-CL-118: "Enter the first day"
+MSG-CL-119: "Enter the first due date"
+MSG-CL-120: "Enter the invoice number"
+MSG-CL-121: "Enter the invoice number to apply the payment to"
+MSG-CL-122: "Enter the promised payment date"
+MSG-CL-123: "Enter the rule code"
+MSG-CL-124: "Enter the rule name"
+MSG-CL-125: "Name the user who receives the escalations"
+MSG-CL-126: "The day of the promise cannot be in the future"
+MSG-CL-127: "The invoice number does not have the expected format"
+MSG-CL-128: "The promised date cannot be before the day of the promise"
+MSG-CL-129: "The rule cannot end before it starts"</t>
         </is>
       </c>
       <c r="M287" s="12" t="inlineStr">
@@ -35055,8 +35055,8 @@
       <c r="L288" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-CL-129: "&lt;Column&gt; '&lt;value&gt;' is not a valid &lt;number, date (yyyy-mm-dd), Y/N value&gt;"
-MSG-CL-130: "&lt;Column&gt; is mandatory"</t>
+MSG-CL-130: "&lt;Column&gt; '&lt;value&gt;' is not a valid &lt;number, date (yyyy-mm-dd), Y/N value&gt;"
+MSG-CL-131: "&lt;Column&gt; is mandatory"</t>
         </is>
       </c>
       <c r="M288" s="12" t="inlineStr">
@@ -35119,15 +35119,15 @@
       <c r="L289" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-CL-131: "&lt;target&gt; does not handle escalations"
-MSG-CL-132: "A promise amount needs the promise date"
-MSG-CL-133: "Escalation Level must be one of &lt;&gt;"
-MSG-CL-134: "Escalation Reason must be a code of the escalation reason list"
-MSG-CL-135: "Fill a promise, Escalate = Y or a worklist field"
-MSG-CL-136: "Invoice &lt;invoice&gt; has nothing to collect"
-MSG-CL-137: "Invoice &lt;invoice&gt; is not in the ledger"
-MSG-CL-138: "Name the user in Escalate To for a USER escalation"
-MSG-CL-139: "You are not allowed to escalate accounts"</t>
+MSG-CL-132: "&lt;target&gt; does not handle escalations"
+MSG-CL-133: "A promise amount needs the promise date"
+MSG-CL-134: "Escalation Level must be one of &lt;&gt;"
+MSG-CL-135: "Escalation Reason must be a code of the escalation reason list"
+MSG-CL-136: "Fill a promise, Escalate = Y or a worklist field"
+MSG-CL-137: "Invoice &lt;invoice&gt; has nothing to collect"
+MSG-CL-138: "Invoice &lt;invoice&gt; is not in the ledger"
+MSG-CL-139: "Name the user in Escalate To for a USER escalation"
+MSG-CL-140: "You are not allowed to escalate accounts"</t>
         </is>
       </c>
       <c r="M289" s="12" t="inlineStr">
@@ -35190,13 +35190,13 @@
       <c r="L290" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-CL-140: "You are not permitted to perform this action" (ACCESS_DENIED)
-MSG-CL-141: "The record was changed by another user. Please reload and try again." (CONCURRENT_MODIFICATION)
-MSG-CL-142: "The system could not complete the request. Try again; if it continues, contact support with the reference." (INTERNAL_ERROR)
-MSG-CL-143: "Parameter '&lt;name&gt;' has an invalid value" (MALFORMED_REQUEST)
-MSG-CL-144: "Required parameter '&lt;parameter name&gt;' is missing" (MALFORMED_REQUEST)
-MSG-CL-145: "The uploaded file is too large" (UPLOAD_TOO_LARGE)
-MSG-CL-146: "Invalid request" (VALIDATION_FAILED)</t>
+MSG-CL-141: "You are not permitted to perform this action" (ACCESS_DENIED)
+MSG-CL-142: "The record was changed by another user. Please reload and try again." (CONCURRENT_MODIFICATION)
+MSG-CL-143: "The system could not complete the request. Try again; if it continues, contact support with the reference." (INTERNAL_ERROR)
+MSG-CL-144: "Parameter '&lt;name&gt;' has an invalid value" (MALFORMED_REQUEST)
+MSG-CL-145: "Required parameter '&lt;parameter name&gt;' is missing" (MALFORMED_REQUEST)
+MSG-CL-146: "The uploaded file is too large" (UPLOAD_TOO_LARGE)
+MSG-CL-147: "Invalid request" (VALIDATION_FAILED)</t>
         </is>
       </c>
       <c r="M290" s="12" t="inlineStr">

</xml_diff>